<commit_message>
Added new files and folderss
</commit_message>
<xml_diff>
--- a/Data/Task 2 Engagement Analysis.xlsx
+++ b/Data/Task 2 Engagement Analysis.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\New folder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\New folder (2)\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B6842A4-BEE2-4955-954E-3B1E8E166105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFB9512D-9EE9-4688-8D92-19A0F6CB3B67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,8 +22,8 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="356" r:id="rId4"/>
-    <pivotCache cacheId="362" r:id="rId5"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
+    <pivotCache cacheId="1" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
@@ -1285,7 +1285,7 @@
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1332,7 +1332,6 @@
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1375,6 +1374,1680 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[Task 2 Engagement Analysis.xlsx]Post!PivotTable60</c:name>
+    <c:fmtId val="0"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-IN"/>
+              <a:t>Engagement_trend</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Post!$U$8</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Sum of Likes</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:multiLvlStrRef>
+              <c:f>Post!$T$9:$T$37</c:f>
+              <c:multiLvlStrCache>
+                <c:ptCount val="24"/>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>Carousel</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>Image</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>Reel</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>Story</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>Text</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>Video</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>Carousel</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>Image</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>Reel</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>Story</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
+                    <c:v>Text</c:v>
+                  </c:pt>
+                  <c:pt idx="11">
+                    <c:v>Video</c:v>
+                  </c:pt>
+                  <c:pt idx="12">
+                    <c:v>Carousel</c:v>
+                  </c:pt>
+                  <c:pt idx="13">
+                    <c:v>Image</c:v>
+                  </c:pt>
+                  <c:pt idx="14">
+                    <c:v>Reel</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>Story</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>Text</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>Video</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>Carousel</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
+                    <c:v>Image</c:v>
+                  </c:pt>
+                  <c:pt idx="20">
+                    <c:v>Reel</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>Story</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>Text</c:v>
+                  </c:pt>
+                  <c:pt idx="23">
+                    <c:v>Video</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>Facebook</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>Instagram</c:v>
+                  </c:pt>
+                  <c:pt idx="12">
+                    <c:v>Twitter</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>YouTube</c:v>
+                  </c:pt>
+                </c:lvl>
+              </c:multiLvlStrCache>
+            </c:multiLvlStrRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Post!$U$9:$U$37</c:f>
+              <c:numCache>
+                <c:formatCode>_ * #,##0.0_ ;_ * \-#,##0.0_ ;_ * "-"??_ ;_ @_ </c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>44476</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>71602</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>36368</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>29405</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>31963</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>28947</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>43948</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>34202</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>32148</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>42649</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>25567</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>25770</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>48649</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>43761</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>27029</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>20466</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>31899</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>29593</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>24926</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>23903</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>32400</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>31968</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>27067</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>31285</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-FE75-4F80-AC68-A50CE7940F52}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Post!$V$8</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Sum of Shares</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:multiLvlStrRef>
+              <c:f>Post!$T$9:$T$37</c:f>
+              <c:multiLvlStrCache>
+                <c:ptCount val="24"/>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>Carousel</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>Image</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>Reel</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>Story</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>Text</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>Video</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>Carousel</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>Image</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>Reel</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>Story</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
+                    <c:v>Text</c:v>
+                  </c:pt>
+                  <c:pt idx="11">
+                    <c:v>Video</c:v>
+                  </c:pt>
+                  <c:pt idx="12">
+                    <c:v>Carousel</c:v>
+                  </c:pt>
+                  <c:pt idx="13">
+                    <c:v>Image</c:v>
+                  </c:pt>
+                  <c:pt idx="14">
+                    <c:v>Reel</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>Story</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>Text</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>Video</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>Carousel</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
+                    <c:v>Image</c:v>
+                  </c:pt>
+                  <c:pt idx="20">
+                    <c:v>Reel</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>Story</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>Text</c:v>
+                  </c:pt>
+                  <c:pt idx="23">
+                    <c:v>Video</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>Facebook</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>Instagram</c:v>
+                  </c:pt>
+                  <c:pt idx="12">
+                    <c:v>Twitter</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>YouTube</c:v>
+                  </c:pt>
+                </c:lvl>
+              </c:multiLvlStrCache>
+            </c:multiLvlStrRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Post!$V$9:$V$37</c:f>
+              <c:numCache>
+                <c:formatCode>_ * #,##0.0_ ;_ * \-#,##0.0_ ;_ * "-"??_ ;_ @_ </c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>7400</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12904</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5964</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4950</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4792</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3171</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6975</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5286</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8110</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10049</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5112</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5912</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5791</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>7110</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>4550</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>5090</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>4861</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>6326</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>6305</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>4310</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>4577</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>3866</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>3928</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>5586</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-FE75-4F80-AC68-A50CE7940F52}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Post!$W$8</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Sum of Comments</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:multiLvlStrRef>
+              <c:f>Post!$T$9:$T$37</c:f>
+              <c:multiLvlStrCache>
+                <c:ptCount val="24"/>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>Carousel</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>Image</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>Reel</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>Story</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>Text</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>Video</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>Carousel</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>Image</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>Reel</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>Story</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
+                    <c:v>Text</c:v>
+                  </c:pt>
+                  <c:pt idx="11">
+                    <c:v>Video</c:v>
+                  </c:pt>
+                  <c:pt idx="12">
+                    <c:v>Carousel</c:v>
+                  </c:pt>
+                  <c:pt idx="13">
+                    <c:v>Image</c:v>
+                  </c:pt>
+                  <c:pt idx="14">
+                    <c:v>Reel</c:v>
+                  </c:pt>
+                  <c:pt idx="15">
+                    <c:v>Story</c:v>
+                  </c:pt>
+                  <c:pt idx="16">
+                    <c:v>Text</c:v>
+                  </c:pt>
+                  <c:pt idx="17">
+                    <c:v>Video</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>Carousel</c:v>
+                  </c:pt>
+                  <c:pt idx="19">
+                    <c:v>Image</c:v>
+                  </c:pt>
+                  <c:pt idx="20">
+                    <c:v>Reel</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>Story</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>Text</c:v>
+                  </c:pt>
+                  <c:pt idx="23">
+                    <c:v>Video</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>Facebook</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>Instagram</c:v>
+                  </c:pt>
+                  <c:pt idx="12">
+                    <c:v>Twitter</c:v>
+                  </c:pt>
+                  <c:pt idx="18">
+                    <c:v>YouTube</c:v>
+                  </c:pt>
+                </c:lvl>
+              </c:multiLvlStrCache>
+            </c:multiLvlStrRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Post!$W$9:$W$37</c:f>
+              <c:numCache>
+                <c:formatCode>_ * #,##0.0_ ;_ * \-#,##0.0_ ;_ * "-"??_ ;_ @_ </c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>4589</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6495</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3353</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3223</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3377</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2263</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3890</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2655</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3386</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3846</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1946</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2128</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>3607</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>5125</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1913</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>3026</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>3910</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>3299</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2422</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2077</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2668</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2012</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>1052</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2589</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-FE75-4F80-AC68-A50CE7940F52}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="407476223"/>
+        <c:axId val="407475743"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="407476223"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="407475743"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="407475743"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="_ * #,##0.0_ ;_ * \-#,##0.0_ ;_ * &quot;-&quot;??_ ;_ @_ " sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="407476223"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>157655</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>140138</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>932793</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>157655</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8B696B12-ACF5-4677-6896-F44E22FB69A0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -12432,7 +14105,375 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{205FAF1C-51DB-492D-83E8-A47F5CD8E358}" name="PivotTable63" cacheId="362" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E6790887-A970-4201-A140-90AD198946F8}" name="PivotTable61" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="T57:U88" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="16">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="3"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="10" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="4"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="3"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="13"/>
+    <field x="14"/>
+  </rowFields>
+  <rowItems count="31">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average of Clicks" fld="12" subtotal="average" baseField="4" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D823DD85-4238-47F1-BE15-A0CC1FCF1CD4}" name="PivotTable60" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+  <location ref="T8:W37" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="16">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="5">
+        <item x="3"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="3"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="10" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="1"/>
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="29">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+  </colItems>
+  <dataFields count="3">
+    <dataField name="Sum of Likes" fld="5" baseField="0" baseItem="0" numFmtId="164"/>
+    <dataField name="Sum of Shares" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+    <dataField name="Sum of Comments" fld="7" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <chartFormats count="3">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight15" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{205FAF1C-51DB-492D-83E8-A47F5CD8E358}" name="PivotTable63" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="T97:U130" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="16">
     <pivotField showAll="0"/>
@@ -12755,345 +14796,6 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E6790887-A970-4201-A140-90AD198946F8}" name="PivotTable61" cacheId="356" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="T57:U88" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="16">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="3"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="10" showAll="0"/>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="4"/>
-        <item x="1"/>
-        <item x="0"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="3"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item x="5"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="13"/>
-    <field x="14"/>
-  </rowFields>
-  <rowItems count="31">
-    <i>
-      <x/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Average of Clicks" fld="12" subtotal="average" baseField="4" baseItem="0" numFmtId="164"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D823DD85-4238-47F1-BE15-A0CC1FCF1CD4}" name="PivotTable60" cacheId="356" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="T8:W37" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="16">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0" sortType="descending">
-      <items count="5">
-        <item x="3"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="1">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="3"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="10" showAll="0"/>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="1"/>
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="29">
-    <i>
-      <x/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-    <i i="2">
-      <x v="2"/>
-    </i>
-  </colItems>
-  <dataFields count="3">
-    <dataField name="Sum of Likes" fld="5" baseField="0" baseItem="0" numFmtId="164"/>
-    <dataField name="Sum of Shares" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
-    <dataField name="Sum of Comments" fld="7" baseField="0" baseItem="0" numFmtId="164"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight15" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
@@ -13520,14 +15222,14 @@
       <c r="P4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="U4" s="23" t="s">
+      <c r="U4" s="22" t="s">
         <v>369</v>
       </c>
-      <c r="V4" s="24"/>
-      <c r="W4" s="24"/>
-      <c r="X4" s="24"/>
-      <c r="Y4" s="24"/>
-      <c r="Z4" s="24"/>
+      <c r="V4" s="23"/>
+      <c r="W4" s="23"/>
+      <c r="X4" s="23"/>
+      <c r="Y4" s="23"/>
+      <c r="Z4" s="23"/>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -16336,11 +18038,11 @@
       <c r="P52" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="T52" s="25" t="s">
+      <c r="T52" s="24" t="s">
         <v>370</v>
       </c>
-      <c r="U52" s="24"/>
-      <c r="V52" s="24"/>
+      <c r="U52" s="23"/>
+      <c r="V52" s="23"/>
     </row>
     <row r="53" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
@@ -18673,10 +20375,10 @@
       <c r="P94" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T94" s="26" t="s">
+      <c r="T94" s="25" t="s">
         <v>368</v>
       </c>
-      <c r="U94" s="24"/>
+      <c r="U94" s="23"/>
     </row>
     <row r="95" spans="1:21" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
@@ -18890,7 +20592,7 @@
       <c r="T98" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="U98" s="22">
+      <c r="U98">
         <v>239605</v>
       </c>
     </row>
@@ -18946,7 +20648,7 @@
       <c r="T99" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="U99" s="22">
+      <c r="U99">
         <v>43741</v>
       </c>
     </row>
@@ -19002,7 +20704,7 @@
       <c r="T100" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="U100" s="22">
+      <c r="U100">
         <v>11504</v>
       </c>
     </row>
@@ -19058,7 +20760,7 @@
       <c r="T101" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="U101" s="22">
+      <c r="U101">
         <v>26773</v>
       </c>
     </row>
@@ -19116,7 +20818,7 @@
       <c r="T102" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="U102" s="22">
+      <c r="U102">
         <v>36804</v>
       </c>
     </row>
@@ -19174,7 +20876,7 @@
       <c r="T103" s="20" t="s">
         <v>366</v>
       </c>
-      <c r="U103" s="22">
+      <c r="U103">
         <v>120783</v>
       </c>
     </row>
@@ -19230,7 +20932,7 @@
       <c r="T104" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="U104" s="22">
+      <c r="U104">
         <v>227957</v>
       </c>
     </row>
@@ -19286,7 +20988,7 @@
       <c r="T105" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="U105" s="22">
+      <c r="U105">
         <v>10681</v>
       </c>
     </row>
@@ -19344,7 +21046,7 @@
       <c r="T106" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="U106" s="22">
+      <c r="U106">
         <v>38336</v>
       </c>
     </row>
@@ -19400,7 +21102,7 @@
       <c r="T107" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="U107" s="22">
+      <c r="U107">
         <v>25449</v>
       </c>
     </row>
@@ -19458,7 +21160,7 @@
       <c r="T108" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="U108" s="22">
+      <c r="U108">
         <v>54027</v>
       </c>
     </row>
@@ -19516,7 +21218,7 @@
       <c r="T109" s="20" t="s">
         <v>366</v>
       </c>
-      <c r="U109" s="22">
+      <c r="U109">
         <v>99464</v>
       </c>
     </row>
@@ -19574,7 +21276,7 @@
       <c r="T110" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="U110" s="22">
+      <c r="U110">
         <v>210680</v>
       </c>
     </row>
@@ -19632,7 +21334,7 @@
       <c r="T111" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="U111" s="22">
+      <c r="U111">
         <v>8859</v>
       </c>
     </row>
@@ -19690,7 +21392,7 @@
       <c r="T112" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="U112" s="22">
+      <c r="U112">
         <v>33589</v>
       </c>
     </row>
@@ -19748,7 +21450,7 @@
       <c r="T113" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="U113" s="22">
+      <c r="U113">
         <v>27064</v>
       </c>
     </row>
@@ -19804,7 +21506,7 @@
       <c r="T114" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="U114" s="22">
+      <c r="U114">
         <v>31065</v>
       </c>
     </row>
@@ -19862,7 +21564,7 @@
       <c r="T115" s="20" t="s">
         <v>366</v>
       </c>
-      <c r="U115" s="22">
+      <c r="U115">
         <v>110103</v>
       </c>
     </row>
@@ -19920,7 +21622,7 @@
       <c r="T116" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="U116" s="22">
+      <c r="U116">
         <v>184397</v>
       </c>
     </row>
@@ -19976,7 +21678,7 @@
       <c r="T117" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="U117" s="22">
+      <c r="U117">
         <v>34283</v>
       </c>
     </row>
@@ -20034,7 +21736,7 @@
       <c r="T118" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="U118" s="22">
+      <c r="U118">
         <v>28297</v>
       </c>
     </row>
@@ -20090,7 +21792,7 @@
       <c r="T119" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="U119" s="22">
+      <c r="U119">
         <v>13184</v>
       </c>
     </row>
@@ -20146,7 +21848,7 @@
       <c r="T120" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="U120" s="22">
+      <c r="U120">
         <v>23668</v>
       </c>
     </row>
@@ -20204,7 +21906,7 @@
       <c r="T121" s="20" t="s">
         <v>366</v>
       </c>
-      <c r="U121" s="22">
+      <c r="U121">
         <v>84965</v>
       </c>
     </row>
@@ -20262,7 +21964,7 @@
       <c r="T122" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="U122" s="22">
+      <c r="U122">
         <v>175128</v>
       </c>
     </row>
@@ -20320,7 +22022,7 @@
       <c r="T123" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="U123" s="22">
+      <c r="U123">
         <v>20211</v>
       </c>
     </row>
@@ -20378,7 +22080,7 @@
       <c r="T124" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="U124" s="22">
+      <c r="U124">
         <v>12627</v>
       </c>
     </row>
@@ -20434,7 +22136,7 @@
       <c r="T125" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="U125" s="22">
+      <c r="U125">
         <v>25137</v>
       </c>
     </row>
@@ -20490,7 +22192,7 @@
       <c r="T126" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="U126" s="22">
+      <c r="U126">
         <v>32532</v>
       </c>
     </row>
@@ -20546,7 +22248,7 @@
       <c r="T127" s="20" t="s">
         <v>366</v>
       </c>
-      <c r="U127" s="22">
+      <c r="U127">
         <v>84621</v>
       </c>
     </row>
@@ -20604,7 +22306,6 @@
       <c r="T128" s="19" t="s">
         <v>366</v>
       </c>
-      <c r="U128" s="22"/>
     </row>
     <row r="129" spans="1:21" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A129" s="2" t="s">
@@ -20658,7 +22359,6 @@
       <c r="T129" s="20" t="s">
         <v>366</v>
       </c>
-      <c r="U129" s="22"/>
     </row>
     <row r="130" spans="1:21" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
@@ -20712,7 +22412,7 @@
       <c r="T130" s="19" t="s">
         <v>361</v>
       </c>
-      <c r="U130" s="22">
+      <c r="U130">
         <v>1037767</v>
       </c>
     </row>
@@ -30166,6 +31866,7 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
+  <drawing r:id="rId4"/>
 </worksheet>
 </file>
 

</xml_diff>